<commit_message>
feat: increase upload limit to 50MB, update API authentication headers, and initialize distributor rules configuration
</commit_message>
<xml_diff>
--- a/backend/Шаблон.xlsx
+++ b/backend/Шаблон.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>СВОДНЫЙ ПРАЙС ООО "НПФ" МАТЕРИА МЕДИКА ХОЛДИНГ"</t>
   </si>
@@ -49,11 +49,7 @@
     <t xml:space="preserve">    "ФАРМ ЛЮКС ИНВЕСТ"                      994860288                994860299 </t>
   </si>
   <si>
-    <t xml:space="preserve">"AERO PHARM         GROUP"                         998550755                   909777866    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">"DELPHARM"    933837402  998771193
-909388567 </t>
+    <t xml:space="preserve">"DELPHARM"    99 877 1153 </t>
   </si>
   <si>
     <t>Эргоферон №20</t>
@@ -74,10 +70,10 @@
     <t>Ренгалин раствор 100 мл</t>
   </si>
   <si>
-    <t>Тенотен №20</t>
-  </si>
-  <si>
-    <t>Тенотен детский №20</t>
+    <t>Тенотен №40</t>
+  </si>
+  <si>
+    <t>Тенотен детский №40</t>
   </si>
   <si>
     <t>Диваза №100</t>
@@ -115,12 +111,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_-* #,##0.00\ _₽_-;\-* #,##0.00\ _₽_-;_-* &quot;-&quot;??\ _₽_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="38">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,33 +236,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <name val="Calibri"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -274,6 +248,14 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -293,7 +275,37 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -308,22 +320,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -337,28 +341,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
@@ -367,6 +349,43 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -374,59 +393,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -449,6 +415,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -461,7 +433,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -473,13 +445,127 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -491,73 +577,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -569,61 +589,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -717,16 +683,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -761,6 +718,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -778,11 +746,18 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
+      <top/>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -801,167 +776,158 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="34" fillId="23" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="32" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1042,29 +1008,12 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="14" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1419,7 +1368,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="8.87826086956522" defaultRowHeight="20.15"/>
   <cols>
     <col min="1" max="1" width="6.05217391304348" style="1" customWidth="1"/>
@@ -1434,21 +1383,20 @@
     <col min="13" max="13" width="12.104347826087" style="1" customWidth="1"/>
     <col min="14" max="14" width="11.5652173913043" style="1" customWidth="1"/>
     <col min="15" max="15" width="12.2347826086957" style="1" customWidth="1"/>
-    <col min="16" max="16" width="12.3739130434783" style="1" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="13.3130434782609" style="1" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="20.3130434782609" style="1" customWidth="1"/>
-    <col min="19" max="19" width="8.4695652173913" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.87826086956522" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="45.4695652173913" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="0.669565217391304" style="1" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="1.34782608695652" style="3" customWidth="1"/>
-    <col min="24" max="24" width="5.24347826086957" style="1" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="2.28695652173913" style="1" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="8.87826086956522" style="1" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="37.5304347826087" style="6" customWidth="1"/>
-    <col min="28" max="28" width="25.8260869565217" style="6" customWidth="1"/>
-    <col min="29" max="29" width="15.7391304347826" style="1" customWidth="1"/>
-    <col min="30" max="16384" width="8.87826086956522" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20.3130434782609" style="1" customWidth="1"/>
+    <col min="17" max="17" width="8.4695652173913" style="1" customWidth="1"/>
+    <col min="18" max="18" width="8.87826086956522" style="1" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="45.4695652173913" style="1" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="0.669565217391304" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="1.34782608695652" style="3" customWidth="1"/>
+    <col min="22" max="22" width="5.24347826086957" style="1" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="2.28695652173913" style="1" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="8.87826086956522" style="1" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="37.5304347826087" style="6" customWidth="1"/>
+    <col min="26" max="26" width="25.8260869565217" style="6" customWidth="1"/>
+    <col min="27" max="27" width="15.7391304347826" style="1" customWidth="1"/>
+    <col min="28" max="16382" width="8.87826086956522" style="1" customWidth="1"/>
+    <col min="16383" max="16384" width="8.87826086956522" style="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.6" customHeight="1"/>
@@ -1462,7 +1410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="15" customHeight="1" spans="1:18">
+    <row r="4" s="1" customFormat="1" ht="15" customHeight="1" spans="1:16">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1499,12 +1447,8 @@
       <c r="P4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="9" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="5" s="2" customFormat="1" ht="87" customHeight="1" spans="1:18">
+    <row r="5" s="2" customFormat="1" ht="87" customHeight="1" spans="1:16">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="C5" s="12"/>
@@ -1520,11 +1464,9 @@
       <c r="M5" s="13"/>
       <c r="N5" s="12"/>
       <c r="O5" s="13"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="11"/>
+      <c r="P5" s="34"/>
     </row>
-    <row r="6" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:18">
+    <row r="6" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
       <c r="A6" s="14"/>
       <c r="B6" s="9"/>
       <c r="C6" s="15">
@@ -1567,21 +1509,15 @@
         <v>1</v>
       </c>
       <c r="P6" s="15">
-        <v>0.25</v>
-      </c>
-      <c r="Q6" s="15">
         <v>1</v>
       </c>
-      <c r="R6" s="35">
-        <v>100</v>
-      </c>
     </row>
-    <row r="7" ht="39" customHeight="1" spans="1:18">
+    <row r="7" ht="39" customHeight="1" spans="1:16">
       <c r="A7" s="16">
         <v>1</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="18">
         <v>47059</v>
@@ -1616,24 +1552,22 @@
       <c r="M7" s="20">
         <v>51360</v>
       </c>
-      <c r="N7" s="34">
+      <c r="N7" s="35">
         <v>47070</v>
       </c>
-      <c r="O7" s="34">
+      <c r="O7" s="35">
         <v>46128</v>
       </c>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="20"/>
-      <c r="R7" s="36">
+      <c r="P7" s="20">
         <v>46683</v>
       </c>
     </row>
-    <row r="8" ht="34.9" customHeight="1" spans="1:18">
+    <row r="8" ht="34.9" customHeight="1" spans="1:16">
       <c r="A8" s="16">
         <v>2</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="20">
         <v>34810</v>
@@ -1675,17 +1609,13 @@
         <v>34125</v>
       </c>
       <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="36">
-        <v>34297</v>
-      </c>
     </row>
-    <row r="9" ht="39" customHeight="1" spans="1:18">
+    <row r="9" ht="39" customHeight="1" spans="1:16">
       <c r="A9" s="16">
         <v>3</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="18">
         <v>42238</v>
@@ -1726,16 +1656,14 @@
       <c r="O9" s="29">
         <v>42604</v>
       </c>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="29"/>
-      <c r="R9" s="37"/>
+      <c r="P9" s="36"/>
     </row>
-    <row r="10" ht="33.75" customHeight="1" spans="1:18">
+    <row r="10" ht="33.75" customHeight="1" spans="1:16">
       <c r="A10" s="16">
         <v>4</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="18">
         <v>34014</v>
@@ -1773,21 +1701,19 @@
       <c r="N10" s="20">
         <v>34025</v>
       </c>
-      <c r="O10" s="34">
+      <c r="O10" s="35">
         <v>33344</v>
       </c>
-      <c r="P10" s="29"/>
-      <c r="Q10" s="29"/>
-      <c r="R10" s="38">
+      <c r="P10" s="29">
         <v>33344</v>
       </c>
     </row>
-    <row r="11" ht="33.6" customHeight="1" spans="1:18">
+    <row r="11" ht="33.6" customHeight="1" spans="1:16">
       <c r="A11" s="16">
         <v>5</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="18"/>
       <c r="D11" s="18"/>
@@ -1818,24 +1744,22 @@
       <c r="M11" s="29">
         <v>30626</v>
       </c>
-      <c r="N11" s="34">
+      <c r="N11" s="35">
         <v>29594</v>
       </c>
-      <c r="O11" s="34">
+      <c r="O11" s="35">
         <v>29002</v>
       </c>
-      <c r="P11" s="29"/>
-      <c r="Q11" s="29"/>
-      <c r="R11" s="36">
+      <c r="P11" s="20">
         <v>31000</v>
       </c>
     </row>
-    <row r="12" ht="33.75" customHeight="1" spans="1:18">
+    <row r="12" ht="33.75" customHeight="1" spans="1:16">
       <c r="A12" s="16">
         <v>6</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="18">
         <v>36104</v>
@@ -1870,22 +1794,20 @@
       <c r="M12" s="23">
         <v>37918</v>
       </c>
-      <c r="N12" s="34">
+      <c r="N12" s="35">
         <v>36115</v>
       </c>
-      <c r="O12" s="34">
+      <c r="O12" s="35">
         <v>35393</v>
       </c>
-      <c r="P12" s="29"/>
-      <c r="Q12" s="29"/>
-      <c r="R12" s="39"/>
+      <c r="P12" s="25"/>
     </row>
-    <row r="13" ht="34.9" customHeight="1" spans="1:18">
+    <row r="13" ht="34.9" customHeight="1" spans="1:16">
       <c r="A13" s="16">
         <v>7</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="18">
         <v>34169</v>
@@ -1919,15 +1841,13 @@
       <c r="N13" s="20"/>
       <c r="O13" s="20"/>
       <c r="P13" s="20"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="36"/>
     </row>
-    <row r="14" ht="31.15" customHeight="1" spans="1:18">
+    <row r="14" ht="31.15" customHeight="1" spans="1:16">
       <c r="A14" s="16">
         <v>8</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="18">
         <v>34689</v>
@@ -1958,24 +1878,22 @@
       <c r="M14" s="20">
         <v>34931</v>
       </c>
-      <c r="N14" s="34">
+      <c r="N14" s="35">
         <v>34700</v>
       </c>
-      <c r="O14" s="34">
+      <c r="O14" s="35">
         <v>34006</v>
       </c>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="36">
+      <c r="P14" s="20">
         <v>34006</v>
       </c>
     </row>
-    <row r="15" ht="30.6" customHeight="1" spans="1:18">
+    <row r="15" ht="30.6" customHeight="1" spans="1:16">
       <c r="A15" s="16">
         <v>9</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
@@ -2003,15 +1921,13 @@
       <c r="N15" s="23"/>
       <c r="O15" s="23"/>
       <c r="P15" s="23"/>
-      <c r="Q15" s="30"/>
-      <c r="R15" s="40"/>
     </row>
-    <row r="16" ht="29.45" customHeight="1" spans="1:18">
+    <row r="16" ht="29.45" customHeight="1" spans="1:16">
       <c r="A16" s="16">
         <v>10</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23"/>
@@ -2035,15 +1951,13 @@
       <c r="N16" s="23"/>
       <c r="O16" s="23"/>
       <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="40"/>
     </row>
-    <row r="17" ht="27.6" customHeight="1" spans="1:18">
+    <row r="17" ht="27.6" customHeight="1" spans="1:16">
       <c r="A17" s="24">
         <v>11</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="25"/>
@@ -2059,15 +1973,13 @@
       <c r="N17" s="25"/>
       <c r="O17" s="25"/>
       <c r="P17" s="25"/>
-      <c r="Q17" s="25"/>
-      <c r="R17" s="39"/>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:18">
+    <row r="18" ht="30" customHeight="1" spans="1:16">
       <c r="A18" s="16">
         <v>12</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
@@ -2095,15 +2007,13 @@
         <v>68764</v>
       </c>
       <c r="P18" s="20"/>
-      <c r="Q18" s="20"/>
-      <c r="R18" s="36"/>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:18">
+    <row r="19" ht="30" customHeight="1" spans="1:16">
       <c r="A19" s="16">
         <v>13</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="18"/>
@@ -2118,16 +2028,14 @@
       <c r="M19" s="20"/>
       <c r="N19" s="26"/>
       <c r="O19" s="20"/>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="26"/>
-      <c r="R19" s="36"/>
+      <c r="P19" s="20"/>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="1:18">
+    <row r="20" ht="30" customHeight="1" spans="1:16">
       <c r="A20" s="16">
         <v>14</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -2148,18 +2056,16 @@
       <c r="M20" s="20">
         <v>17725</v>
       </c>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
       <c r="P20" s="20"/>
-      <c r="Q20" s="20"/>
-      <c r="R20" s="36"/>
     </row>
-    <row r="21" ht="33.6" customHeight="1" spans="1:18">
+    <row r="21" ht="33.6" customHeight="1" spans="1:16">
       <c r="A21" s="16">
         <v>15</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C21" s="18">
         <v>15085</v>
@@ -2196,16 +2102,14 @@
       <c r="O21" s="20">
         <v>14794</v>
       </c>
-      <c r="P21" s="20"/>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="41"/>
+      <c r="P21" s="26"/>
     </row>
-    <row r="22" ht="30.6" customHeight="1" spans="1:18">
+    <row r="22" ht="30.6" customHeight="1" spans="1:16">
       <c r="A22" s="16">
         <v>16</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C22" s="23"/>
       <c r="D22" s="23"/>
@@ -2222,18 +2126,16 @@
       <c r="K22" s="26"/>
       <c r="L22" s="26"/>
       <c r="M22" s="26"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
       <c r="P22" s="26"/>
-      <c r="Q22" s="26"/>
-      <c r="R22" s="41"/>
     </row>
-    <row r="23" ht="30.6" customHeight="1" spans="1:18">
+    <row r="23" ht="30.6" customHeight="1" spans="1:16">
       <c r="A23" s="16">
         <v>17</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
@@ -2254,20 +2156,18 @@
       <c r="K23" s="26"/>
       <c r="L23" s="26"/>
       <c r="M23" s="26"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="34"/>
-      <c r="P23" s="20"/>
-      <c r="Q23" s="20"/>
-      <c r="R23" s="41">
+      <c r="N23" s="35"/>
+      <c r="O23" s="35"/>
+      <c r="P23" s="26">
         <v>14214</v>
       </c>
     </row>
-    <row r="24" ht="26.45" customHeight="1" spans="1:18">
+    <row r="24" ht="26.45" customHeight="1" spans="1:16">
       <c r="A24" s="16">
         <v>18</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" s="26"/>
       <c r="D24" s="26"/>
@@ -2283,14 +2183,12 @@
       <c r="N24" s="26"/>
       <c r="O24" s="26"/>
       <c r="P24" s="26"/>
-      <c r="Q24" s="26"/>
-      <c r="R24" s="26"/>
     </row>
     <row r="26" ht="19.5" customHeight="1"/>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A3:R3"/>
+  <mergeCells count="16">
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A3:P3"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="B4:B5"/>
@@ -2298,10 +2196,9 @@
     <mergeCell ref="H25:H26"/>
     <mergeCell ref="J25:J26"/>
     <mergeCell ref="K4:K5"/>
-    <mergeCell ref="R4:R5"/>
+    <mergeCell ref="P4:P5"/>
     <mergeCell ref="L4:M5"/>
     <mergeCell ref="N4:O5"/>
-    <mergeCell ref="P4:Q5"/>
     <mergeCell ref="C4:D5"/>
     <mergeCell ref="E4:F5"/>
     <mergeCell ref="G4:H5"/>

</xml_diff>

<commit_message>
chore: remove unused configuration file
</commit_message>
<xml_diff>
--- a/backend/Шаблон.xlsx
+++ b/backend/Шаблон.xlsx
@@ -58,7 +58,7 @@
     <t>Анаферон детский №20</t>
   </si>
   <si>
-    <t>Анаферон детский №20 капли</t>
+    <t>Анаферон детский капли №1</t>
   </si>
   <si>
     <t>Анаферон №20</t>
@@ -67,7 +67,7 @@
     <t>Ренгалин таб №20</t>
   </si>
   <si>
-    <t>Ренгалин раствор 100 мл</t>
+    <t>Ренгалин раствор 100 мл №1</t>
   </si>
   <si>
     <t>Тенотен №40</t>
@@ -111,9 +111,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_-* #,##0.00\ _₽_-;\-* #,##0.00\ _₽_-;_-* &quot;-&quot;??\ _₽_-;_-@_-"/>
   </numFmts>
   <fonts count="38">
@@ -252,6 +252,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
@@ -274,17 +282,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -303,6 +313,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
@@ -311,14 +328,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
@@ -326,8 +335,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -341,11 +351,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -358,21 +381,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -385,14 +393,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -415,97 +415,169 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -517,79 +589,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -679,11 +679,46 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -699,6 +734,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -720,201 +770,151 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="32" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1372,7 +1372,7 @@
   <sheetFormatPr defaultColWidth="8.87826086956522" defaultRowHeight="20.15"/>
   <cols>
     <col min="1" max="1" width="6.05217391304348" style="1" customWidth="1"/>
-    <col min="2" max="2" width="35.5130434782609" style="4" customWidth="1"/>
+    <col min="2" max="2" width="37.8521739130435" style="4" customWidth="1"/>
     <col min="3" max="3" width="11.295652173913" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.0260869565217" style="5" customWidth="1"/>
     <col min="5" max="5" width="11.9739130434783" style="1" customWidth="1"/>

</xml_diff>